<commit_message>
Record successful hosted CI and approved public project planning evidence
</commit_message>
<xml_diff>
--- a/docs/Project-Plan.xlsx
+++ b/docs/Project-Plan.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly plan" sheetId="1" r:id="Rb0268146970e438a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Annual roadmap" sheetId="2" r:id="Re0459418dbcd43a5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly plan" sheetId="1" r:id="Rc643aa0271094538"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Annual roadmap" sheetId="2" r:id="R4793070b7d384370"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -447,7 +447,7 @@
         <x:v>T4</x:v>
       </x:c>
       <x:c r="B8" s="8" t="d">
-        <x:v>2026-10-26T00:00:00.000Z</x:v>
+        <x:v>2026-10-19T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C8" s="7" t="str">
         <x:v>GitHub Actions CI</x:v>
@@ -459,10 +459,10 @@
         <x:v>0.5</x:v>
       </x:c>
       <x:c r="F8" s="7" t="str">
-        <x:v>To Do</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="G8" s="7" t="str">
-        <x:v>Successful run, README badge and screenshot.</x:v>
+        <x:v>Run 40173810937 succeeded; 31 tests, lint and artifacts.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="44" customHeight="1">
@@ -645,23 +645,27 @@
       <x:c r="F20" s="12"/>
       <x:c r="G20" s="12"/>
     </x:row>
-    <x:row r="21" ht="44" customHeight="1">
-      <x:c r="A21" s="7"/>
-      <x:c r="B21" s="7"/>
-      <x:c r="C21" s="7"/>
-      <x:c r="D21" s="7"/>
-      <x:c r="E21" s="7"/>
-      <x:c r="F21" s="7"/>
-      <x:c r="G21" s="7"/>
-    </x:row>
-    <x:row r="22" ht="44" customHeight="1">
-      <x:c r="A22" s="7"/>
-      <x:c r="B22" s="7"/>
-      <x:c r="C22" s="7"/>
-      <x:c r="D22" s="7"/>
-      <x:c r="E22" s="7"/>
-      <x:c r="F22" s="7"/>
-      <x:c r="G22" s="7"/>
+    <x:row r="21" ht="24" customHeight="1">
+      <x:c r="A21" s="12" t="str">
+        <x:v>Trello: https://trello.com/b/9wbc68TD/nd082-azure-ci-cd (publicly readable; T1, T2 and T4 Done).</x:v>
+      </x:c>
+      <x:c r="B21" s="12"/>
+      <x:c r="C21" s="12"/>
+      <x:c r="D21" s="12"/>
+      <x:c r="E21" s="12"/>
+      <x:c r="F21" s="12"/>
+      <x:c r="G21" s="12"/>
+    </x:row>
+    <x:row r="22" ht="24" customHeight="1">
+      <x:c r="A22" s="12" t="str">
+        <x:v>GitHub Actions: https://github.com/djessijorge9-ship-it/nd082-azure-cicd/actions/runs/40173810937</x:v>
+      </x:c>
+      <x:c r="B22" s="12"/>
+      <x:c r="C22" s="12"/>
+      <x:c r="D22" s="12"/>
+      <x:c r="E22" s="12"/>
+      <x:c r="F22" s="12"/>
+      <x:c r="G22" s="12"/>
     </x:row>
     <x:row r="23" ht="44" customHeight="1">
       <x:c r="A23" s="7"/>

</xml_diff>

<commit_message>
Document verified attended Azure delivery and actual published test evidence
</commit_message>
<xml_diff>
--- a/docs/Project-Plan.xlsx
+++ b/docs/Project-Plan.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly plan" sheetId="1" r:id="Rc643aa0271094538"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Annual roadmap" sheetId="2" r:id="R4793070b7d384370"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly plan" sheetId="1" r:id="R02b433281e11419f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Annual roadmap" sheetId="2" r:id="R0fad02d98c564564"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -416,7 +416,7 @@
         <x:v>Done</x:v>
       </x:c>
       <x:c r="G6" s="7" t="str">
-        <x:v>Added schema tests and reproduced matching-version model.</x:v>
+        <x:v>48 tests pass; matching-version model reproduced and validated.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="44" customHeight="1">
@@ -436,10 +436,10 @@
         <x:v>0.5</x:v>
       </x:c>
       <x:c r="F7" s="7" t="str">
-        <x:v>To Do</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="G7" s="7" t="str">
-        <x:v>Capture clone, build and separate test screenshots.</x:v>
+        <x:v>Completed 25 Oct: 48 tests, lint 10/10, exit 0 in actual Cloud Shell.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="44" customHeight="1">
@@ -462,7 +462,7 @@
         <x:v>Done</x:v>
       </x:c>
       <x:c r="G8" s="7" t="str">
-        <x:v>Run 40173810937 succeeded; 31 tests, lint and artifacts.</x:v>
+        <x:v>Run 40189164258 succeeded at source 3fc837; 48 tests and artifacts.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="44" customHeight="1">
@@ -482,10 +482,10 @@
         <x:v>0.5</x:v>
       </x:c>
       <x:c r="F9" s="7" t="str">
-        <x:v>To Do</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="G9" s="7" t="str">
-        <x:v>Run commands.sh; actual HTTPS prediction and log stream.</x:v>
+        <x:v>F1 deployed; genuine HTTPS single/batch predictions and matching runtime logs.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="44" customHeight="1">
@@ -496,7 +496,7 @@
         <x:v>2026-11-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C10" s="7" t="str">
-        <x:v>Azure Pipelines automatic delivery</x:v>
+        <x:v>Attended Azure Pipelines delivery</x:v>
       </x:c>
       <x:c r="D10" s="9" t="n">
         <x:v>1</x:v>
@@ -505,10 +505,10 @@
         <x:v>1.5</x:v>
       </x:c>
       <x:c r="F10" s="7" t="str">
-        <x:v>To Do</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="G10" s="7" t="str">
-        <x:v>Permitted existing connection, test and two deployment runs.</x:v>
+        <x:v>Run 3 passed: 48 published tests, Entra deployment, smoke and cleanup; manual auth.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="44" customHeight="1">
@@ -625,7 +625,7 @@
     </x:row>
     <x:row r="19" ht="24" customHeight="1">
       <x:c r="A19" s="12" t="str">
-        <x:v>Original estimates were preparation targets. Revised estimates include model compatibility and cloud-connection risk.</x:v>
+        <x:v>Original estimates were preparation targets. Revised estimates include model compatibility and provider connection constraints and attended authentication.</x:v>
       </x:c>
       <x:c r="B19" s="12"/>
       <x:c r="C19" s="12"/>
@@ -647,7 +647,7 @@
     </x:row>
     <x:row r="21" ht="24" customHeight="1">
       <x:c r="A21" s="12" t="str">
-        <x:v>Trello: https://trello.com/b/9wbc68TD/nd082-azure-ci-cd (publicly readable; T1, T2 and T4 Done).</x:v>
+        <x:v>Trello: https://trello.com/b/9wbc68TD/nd082-azure-ci-cd (publicly readable; T1–T6 Done, T7/T8 pending).</x:v>
       </x:c>
       <x:c r="B21" s="12"/>
       <x:c r="C21" s="12"/>
@@ -658,7 +658,7 @@
     </x:row>
     <x:row r="22" ht="24" customHeight="1">
       <x:c r="A22" s="12" t="str">
-        <x:v>GitHub Actions: https://github.com/djessijorge9-ship-it/nd082-azure-cicd/actions/runs/40173810937</x:v>
+        <x:v>GitHub Actions: https://github.com/djessijorge9-ship-it/nd082-azure-cicd/actions/runs/40189164258</x:v>
       </x:c>
       <x:c r="B22" s="12"/>
       <x:c r="C22" s="12"/>

</xml_diff>

<commit_message>
Record verified resource cleanup and historical deployment status
</commit_message>
<xml_diff>
--- a/docs/Project-Plan.xlsx
+++ b/docs/Project-Plan.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly plan" sheetId="1" r:id="R02b433281e11419f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Annual roadmap" sheetId="2" r:id="R0fad02d98c564564"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly plan" sheetId="1" r:id="Rcb304c03a25445d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Annual roadmap" sheetId="2" r:id="Rc534a2e212164ee0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -341,7 +341,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="2" t="str">
-        <x:v>As of 25 October 2026. Revised plan remains open until cloud evidence is complete.</x:v>
+        <x:v>As of 25 October 2026. Cloud evidence complete; revised plan remains open for video publication/handoff.</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -528,10 +528,10 @@
         <x:v>0.5</x:v>
       </x:c>
       <x:c r="F11" s="7" t="str">
-        <x:v>To Do</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="G11" s="7" t="str">
-        <x:v>Board with To Do / In Progress / Done; genuine screenshots.</x:v>
+        <x:v>Actual native screenshots, trace and video validation assembled.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="44" customHeight="1">
@@ -647,7 +647,7 @@
     </x:row>
     <x:row r="21" ht="24" customHeight="1">
       <x:c r="A21" s="12" t="str">
-        <x:v>Trello: https://trello.com/b/9wbc68TD/nd082-azure-ci-cd (publicly readable; T1–T6 Done, T7/T8 pending).</x:v>
+        <x:v>Trello: https://trello.com/b/9wbc68TD/nd082-azure-ci-cd (publicly readable; T1–T7 Done, T8 publication pending).</x:v>
       </x:c>
       <x:c r="B21" s="12"/>
       <x:c r="C21" s="12"/>

</xml_diff>